<commit_message>
Implemented data-driven login test using Excel and TestNG DataProvider
</commit_message>
<xml_diff>
--- a/testData/OpenCart_LoginData.xlsx
+++ b/testData/OpenCart_LoginData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
   <si>
     <t>username</t>
   </si>
@@ -31,19 +31,13 @@
     <t>Valid</t>
   </si>
   <si>
-    <t>lakshmi@yahoo.com</t>
-  </si>
-  <si>
     <t>Invalid</t>
   </si>
   <si>
-    <t>laksh@yahoo.com</t>
+    <t>nihalmadvi2001@gmail.com</t>
   </si>
   <si>
-    <t>vdbhegdr</t>
-  </si>
-  <si>
-    <t>laks@yahoo.com</t>
+    <t>nihalmadvi1</t>
   </si>
   <si>
     <t>xyz</t>
@@ -111,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -128,10 +122,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -380,43 +377,43 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" s="6">
         <v>123.0</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>4</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>13</v>
+      <c r="A6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>5</v>

</xml_diff>